<commit_message>
Version 1.3: Enhanced candidate dashboard
</commit_message>
<xml_diff>
--- a/4063.T_settings.xlsx
+++ b/4063.T_settings.xlsx
@@ -509,22 +509,22 @@
         <v>42.85714285714285</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.802726560579659</v>
+        <v>-2.802701754742849</v>
       </c>
       <c r="G2" t="n">
         <v>14</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.2001947543271185</v>
+        <v>-0.2001929824816321</v>
       </c>
       <c r="I2" t="n">
-        <v>-28027.26560579659</v>
+        <v>-28027.01754742849</v>
       </c>
       <c r="J2" t="n">
-        <v>971972.7343942034</v>
+        <v>971972.9824525715</v>
       </c>
       <c r="K2" t="n">
-        <v>29095.98258296405</v>
+        <v>29095.98746484961</v>
       </c>
       <c r="L2" t="n">
         <v>10.07142857142857</v>
@@ -557,28 +557,28 @@
         <v>43.75</v>
       </c>
       <c r="F3" t="n">
-        <v>-4.060038097188087</v>
+        <v>-4.060025009293854</v>
       </c>
       <c r="G3" t="n">
         <v>16</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.2537523810742554</v>
+        <v>-0.2537515630808659</v>
       </c>
       <c r="I3" t="n">
-        <v>-40600.38097188086</v>
+        <v>-40600.25009293854</v>
       </c>
       <c r="J3" t="n">
-        <v>959399.6190281191</v>
+        <v>959399.7499070615</v>
       </c>
       <c r="K3" t="n">
-        <v>33766.08661664277</v>
+        <v>33766.08783512768</v>
       </c>
       <c r="L3" t="n">
         <v>8.75</v>
       </c>
       <c r="M3" t="n">
-        <v>20.98950193418336</v>
+        <v>20.98949962662807</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -605,28 +605,28 @@
         <v>43.75</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.578523201229308</v>
+        <v>-4.578520414521766</v>
       </c>
       <c r="G4" t="n">
         <v>16</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2861577000768317</v>
+        <v>-0.2861575259076104</v>
       </c>
       <c r="I4" t="n">
-        <v>-45785.23201229307</v>
+        <v>-45785.20414521766</v>
       </c>
       <c r="J4" t="n">
-        <v>954214.7679877069</v>
+        <v>954214.7958547823</v>
       </c>
       <c r="K4" t="n">
-        <v>33698.98857206266</v>
+        <v>33698.98834790901</v>
       </c>
       <c r="L4" t="n">
         <v>9.1875</v>
       </c>
       <c r="M4" t="n">
-        <v>21.41649570713797</v>
+        <v>21.4165018372532</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -653,28 +653,28 @@
         <v>40</v>
       </c>
       <c r="F5" t="n">
-        <v>-10.24091592058061</v>
+        <v>-10.24088338975383</v>
       </c>
       <c r="G5" t="n">
         <v>15</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.6827277280387073</v>
+        <v>-0.6827255593169217</v>
       </c>
       <c r="I5" t="n">
-        <v>-102409.1592058061</v>
+        <v>-102408.8338975383</v>
       </c>
       <c r="J5" t="n">
-        <v>897590.8407941939</v>
+        <v>897591.1661024617</v>
       </c>
       <c r="K5" t="n">
-        <v>30344.82633229367</v>
+        <v>30344.83288075211</v>
       </c>
       <c r="L5" t="n">
         <v>8.4</v>
       </c>
       <c r="M5" t="n">
-        <v>20.38854898124413</v>
+        <v>20.38854665620392</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -701,28 +701,28 @@
         <v>41.17647058823529</v>
       </c>
       <c r="F6" t="n">
-        <v>-10.8961164887405</v>
+        <v>-10.89609331755272</v>
       </c>
       <c r="G6" t="n">
         <v>17</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.6409480287494411</v>
+        <v>-0.640946665738395</v>
       </c>
       <c r="I6" t="n">
-        <v>-108961.164887405</v>
+        <v>-108960.9331755271</v>
       </c>
       <c r="J6" t="n">
-        <v>891038.835112595</v>
+        <v>891039.0668244729</v>
       </c>
       <c r="K6" t="n">
-        <v>33934.52760490893</v>
+        <v>33934.53271168897</v>
       </c>
       <c r="L6" t="n">
         <v>7.588235294117647</v>
       </c>
       <c r="M6" t="n">
-        <v>22.52191591986853</v>
+        <v>22.52191365706845</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -749,28 +749,28 @@
         <v>40</v>
       </c>
       <c r="F7" t="n">
-        <v>-11.44125619710014</v>
+        <v>-11.44125905477309</v>
       </c>
       <c r="G7" t="n">
         <v>15</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.7627504131400096</v>
+        <v>-0.7627506036515395</v>
       </c>
       <c r="I7" t="n">
-        <v>-114412.5619710014</v>
+        <v>-114412.5905477309</v>
       </c>
       <c r="J7" t="n">
-        <v>885587.4380289986</v>
+        <v>885587.4094522691</v>
       </c>
       <c r="K7" t="n">
-        <v>29853.80125966046</v>
+        <v>29853.80066904918</v>
       </c>
       <c r="L7" t="n">
         <v>11.66666666666667</v>
       </c>
       <c r="M7" t="n">
-        <v>21.41649570713796</v>
+        <v>21.41650183725321</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -797,28 +797,28 @@
         <v>38.88888888888889</v>
       </c>
       <c r="F8" t="n">
-        <v>-11.77904887004513</v>
+        <v>-11.77903666878252</v>
       </c>
       <c r="G8" t="n">
         <v>18</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.6543916038913964</v>
+        <v>-0.6543909260434733</v>
       </c>
       <c r="I8" t="n">
-        <v>-117790.4887004513</v>
+        <v>-117790.3666878252</v>
       </c>
       <c r="J8" t="n">
-        <v>882209.5112995487</v>
+        <v>882209.6333121748</v>
       </c>
       <c r="K8" t="n">
-        <v>34902.96231083123</v>
+        <v>34902.96336306122</v>
       </c>
       <c r="L8" t="n">
         <v>9</v>
       </c>
       <c r="M8" t="n">
-        <v>20.98950193418336</v>
+        <v>20.9894996266281</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -845,28 +845,28 @@
         <v>38.88888888888889</v>
       </c>
       <c r="F9" t="n">
-        <v>-12.25581838420823</v>
+        <v>-12.25581565623217</v>
       </c>
       <c r="G9" t="n">
         <v>18</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.6808787991226793</v>
+        <v>-0.680878647568454</v>
       </c>
       <c r="I9" t="n">
-        <v>-122558.1838420823</v>
+        <v>-122558.1565623217</v>
       </c>
       <c r="J9" t="n">
-        <v>877441.8161579177</v>
+        <v>877441.8434376783</v>
       </c>
       <c r="K9" t="n">
-        <v>34841.26275212373</v>
+        <v>34841.26247766871</v>
       </c>
       <c r="L9" t="n">
         <v>9.388888888888889</v>
       </c>
       <c r="M9" t="n">
-        <v>21.41649570713797</v>
+        <v>21.41650183725323</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
@@ -893,28 +893,28 @@
         <v>25</v>
       </c>
       <c r="F10" t="n">
-        <v>-15.04577286742352</v>
+        <v>-15.04576461638634</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
       </c>
       <c r="H10" t="n">
-        <v>-1.88072160842794</v>
+        <v>-1.880720577048292</v>
       </c>
       <c r="I10" t="n">
-        <v>-150457.7286742352</v>
+        <v>-150457.6461638634</v>
       </c>
       <c r="J10" t="n">
-        <v>849542.2713257648</v>
+        <v>849542.3538361366</v>
       </c>
       <c r="K10" t="n">
-        <v>15064.36446141597</v>
+        <v>15064.36479132166</v>
       </c>
       <c r="L10" t="n">
         <v>4.25</v>
       </c>
       <c r="M10" t="n">
-        <v>17.32612043598923</v>
+        <v>17.32610318247631</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
@@ -941,28 +941,28 @@
         <v>25</v>
       </c>
       <c r="F11" t="n">
-        <v>-15.04577286742352</v>
+        <v>-15.04576461638634</v>
       </c>
       <c r="G11" t="n">
         <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>-1.88072160842794</v>
+        <v>-1.880720577048292</v>
       </c>
       <c r="I11" t="n">
-        <v>-150457.7286742352</v>
+        <v>-150457.6461638634</v>
       </c>
       <c r="J11" t="n">
-        <v>849542.2713257648</v>
+        <v>849542.3538361366</v>
       </c>
       <c r="K11" t="n">
-        <v>15064.36446141597</v>
+        <v>15064.36479132166</v>
       </c>
       <c r="L11" t="n">
         <v>4.25</v>
       </c>
       <c r="M11" t="n">
-        <v>17.32612043598923</v>
+        <v>17.32610318247631</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
@@ -989,28 +989,28 @@
         <v>28.57142857142857</v>
       </c>
       <c r="F12" t="n">
-        <v>-15.63110960558923</v>
+        <v>-15.63110728425528</v>
       </c>
       <c r="G12" t="n">
         <v>7</v>
       </c>
       <c r="H12" t="n">
-        <v>-2.233015657941319</v>
+        <v>-2.233015326322183</v>
       </c>
       <c r="I12" t="n">
-        <v>-156311.0960558923</v>
+        <v>-156311.0728425528</v>
       </c>
       <c r="J12" t="n">
-        <v>843688.9039441077</v>
+        <v>843688.9271574472</v>
       </c>
       <c r="K12" t="n">
-        <v>12810.63815930555</v>
+        <v>12810.6380640939</v>
       </c>
       <c r="L12" t="n">
         <v>5.714285714285714</v>
       </c>
       <c r="M12" t="n">
-        <v>15.63110960558923</v>
+        <v>15.63110728425528</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
@@ -1037,28 +1037,28 @@
         <v>28.57142857142857</v>
       </c>
       <c r="F13" t="n">
-        <v>-15.63110960558923</v>
+        <v>-15.63110728425528</v>
       </c>
       <c r="G13" t="n">
         <v>7</v>
       </c>
       <c r="H13" t="n">
-        <v>-2.233015657941319</v>
+        <v>-2.233015326322183</v>
       </c>
       <c r="I13" t="n">
-        <v>-156311.0960558923</v>
+        <v>-156311.0728425528</v>
       </c>
       <c r="J13" t="n">
-        <v>843688.9039441077</v>
+        <v>843688.9271574472</v>
       </c>
       <c r="K13" t="n">
-        <v>12810.63815930555</v>
+        <v>12810.6380640939</v>
       </c>
       <c r="L13" t="n">
         <v>5.714285714285714</v>
       </c>
       <c r="M13" t="n">
-        <v>15.63110960558923</v>
+        <v>15.63110728425528</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
@@ -1085,28 +1085,28 @@
         <v>28.57142857142857</v>
       </c>
       <c r="F14" t="n">
-        <v>-15.63110960558923</v>
+        <v>-15.63110728425528</v>
       </c>
       <c r="G14" t="n">
         <v>7</v>
       </c>
       <c r="H14" t="n">
-        <v>-2.233015657941319</v>
+        <v>-2.233015326322183</v>
       </c>
       <c r="I14" t="n">
-        <v>-156311.0960558923</v>
+        <v>-156311.0728425528</v>
       </c>
       <c r="J14" t="n">
-        <v>843688.9039441077</v>
+        <v>843688.9271574472</v>
       </c>
       <c r="K14" t="n">
-        <v>12810.63815930555</v>
+        <v>12810.6380640939</v>
       </c>
       <c r="L14" t="n">
         <v>5.714285714285714</v>
       </c>
       <c r="M14" t="n">
-        <v>15.63110960558923</v>
+        <v>15.63110728425528</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -1133,28 +1133,28 @@
         <v>25</v>
       </c>
       <c r="F15" t="n">
-        <v>-15.70415283082771</v>
+        <v>-15.7041536813865</v>
       </c>
       <c r="G15" t="n">
         <v>8</v>
       </c>
       <c r="H15" t="n">
-        <v>-1.963019103853464</v>
+        <v>-1.963019210173312</v>
       </c>
       <c r="I15" t="n">
-        <v>-157041.5283082771</v>
+        <v>-157041.536813865</v>
       </c>
       <c r="J15" t="n">
-        <v>842958.4716917229</v>
+        <v>842958.463186135</v>
       </c>
       <c r="K15" t="n">
-        <v>14986.32280408577</v>
+        <v>14986.32205669587</v>
       </c>
       <c r="L15" t="n">
         <v>5</v>
       </c>
       <c r="M15" t="n">
-        <v>17.96682811633683</v>
+        <v>17.96681979159911</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
@@ -1181,28 +1181,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F16" t="n">
-        <v>-17.4769835836221</v>
+        <v>-17.47697795667928</v>
       </c>
       <c r="G16" t="n">
         <v>15</v>
       </c>
       <c r="H16" t="n">
-        <v>-1.16513223890814</v>
+        <v>-1.165131863778619</v>
       </c>
       <c r="I16" t="n">
-        <v>-174769.835836221</v>
+        <v>-174769.7795667928</v>
       </c>
       <c r="J16" t="n">
-        <v>825230.164163779</v>
+        <v>825230.2204332072</v>
       </c>
       <c r="K16" t="n">
-        <v>28527.87188429123</v>
+        <v>28527.8724449474</v>
       </c>
       <c r="L16" t="n">
         <v>8.866666666666667</v>
       </c>
       <c r="M16" t="n">
-        <v>20.98950193418338</v>
+        <v>20.98949962662808</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
@@ -1229,28 +1229,28 @@
         <v>37.5</v>
       </c>
       <c r="F17" t="n">
-        <v>-17.96191933763932</v>
+        <v>-17.9618794627715</v>
       </c>
       <c r="G17" t="n">
         <v>16</v>
       </c>
       <c r="H17" t="n">
-        <v>-1.122619958602457</v>
+        <v>-1.122617466423219</v>
       </c>
       <c r="I17" t="n">
-        <v>-179619.1933763932</v>
+        <v>-179618.794627715</v>
       </c>
       <c r="J17" t="n">
-        <v>820380.8066236068</v>
+        <v>820381.205372285</v>
       </c>
       <c r="K17" t="n">
-        <v>29975.94529799559</v>
+        <v>29975.95545972505</v>
       </c>
       <c r="L17" t="n">
         <v>7.25</v>
       </c>
       <c r="M17" t="n">
-        <v>21.93261849033902</v>
+        <v>21.93261621039316</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
@@ -1277,28 +1277,28 @@
         <v>36.84210526315789</v>
       </c>
       <c r="F18" t="n">
-        <v>-18.06511909292697</v>
+        <v>-18.06509763149402</v>
       </c>
       <c r="G18" t="n">
         <v>19</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.9507957417329983</v>
+        <v>-0.9507946121838956</v>
       </c>
       <c r="I18" t="n">
-        <v>-180651.1909292697</v>
+        <v>-180650.9763149401</v>
       </c>
       <c r="J18" t="n">
-        <v>819348.8090707303</v>
+        <v>819349.0236850599</v>
       </c>
       <c r="K18" t="n">
-        <v>35057.85109647787</v>
+        <v>35057.8557244558</v>
       </c>
       <c r="L18" t="n">
         <v>7.947368421052632</v>
       </c>
       <c r="M18" t="n">
-        <v>22.52191591986853</v>
+        <v>22.52191365706844</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
@@ -1325,28 +1325,28 @@
         <v>30</v>
       </c>
       <c r="F19" t="n">
-        <v>-18.48307112161624</v>
+        <v>-18.48305929591534</v>
       </c>
       <c r="G19" t="n">
         <v>10</v>
       </c>
       <c r="H19" t="n">
-        <v>-1.848307112161624</v>
+        <v>-1.848305929591534</v>
       </c>
       <c r="I19" t="n">
-        <v>-184830.7112161624</v>
+        <v>-184830.5929591533</v>
       </c>
       <c r="J19" t="n">
-        <v>815169.2887838376</v>
+        <v>815169.4070408467</v>
       </c>
       <c r="K19" t="n">
-        <v>19505.99246240086</v>
+        <v>19505.99428466548</v>
       </c>
       <c r="L19" t="n">
         <v>7.9</v>
       </c>
       <c r="M19" t="n">
-        <v>25.5385874692687</v>
+        <v>25.53859302268384</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
@@ -1373,28 +1373,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F20" t="n">
-        <v>-18.48956489762778</v>
+        <v>-18.48955948939248</v>
       </c>
       <c r="G20" t="n">
         <v>9</v>
       </c>
       <c r="H20" t="n">
-        <v>-2.05439609973642</v>
+        <v>-2.054395498821386</v>
       </c>
       <c r="I20" t="n">
-        <v>-184895.6489762778</v>
+        <v>-184895.5948939248</v>
       </c>
       <c r="J20" t="n">
-        <v>815104.3510237222</v>
+        <v>815104.4051060752</v>
       </c>
       <c r="K20" t="n">
-        <v>16222.69037186876</v>
+        <v>16222.69048683836</v>
       </c>
       <c r="L20" t="n">
         <v>4.333333333333333</v>
       </c>
       <c r="M20" t="n">
-        <v>18.48956489762778</v>
+        <v>18.48955948939248</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
@@ -1421,28 +1421,28 @@
         <v>20</v>
       </c>
       <c r="F21" t="n">
-        <v>-18.9432772065834</v>
+        <v>-18.94322949128189</v>
       </c>
       <c r="G21" t="n">
         <v>10</v>
       </c>
       <c r="H21" t="n">
-        <v>-1.89432772065834</v>
+        <v>-1.894322949128189</v>
       </c>
       <c r="I21" t="n">
-        <v>-189432.772065834</v>
+        <v>-189432.2949128189</v>
       </c>
       <c r="J21" t="n">
-        <v>810567.227934166</v>
+        <v>810567.7050871811</v>
       </c>
       <c r="K21" t="n">
-        <v>18077.71269817773</v>
+        <v>18077.7194609615</v>
       </c>
       <c r="L21" t="n">
         <v>6.5</v>
       </c>
       <c r="M21" t="n">
-        <v>18.9432772065834</v>
+        <v>18.94322949128189</v>
       </c>
       <c r="N21" t="b">
         <v>1</v>
@@ -1469,28 +1469,28 @@
         <v>20</v>
       </c>
       <c r="F22" t="n">
-        <v>-18.9432772065834</v>
+        <v>-18.94322949128189</v>
       </c>
       <c r="G22" t="n">
         <v>10</v>
       </c>
       <c r="H22" t="n">
-        <v>-1.89432772065834</v>
+        <v>-1.894322949128189</v>
       </c>
       <c r="I22" t="n">
-        <v>-189432.772065834</v>
+        <v>-189432.2949128189</v>
       </c>
       <c r="J22" t="n">
-        <v>810567.227934166</v>
+        <v>810567.7050871811</v>
       </c>
       <c r="K22" t="n">
-        <v>18077.71269817773</v>
+        <v>18077.7194609615</v>
       </c>
       <c r="L22" t="n">
         <v>6.5</v>
       </c>
       <c r="M22" t="n">
-        <v>18.9432772065834</v>
+        <v>18.94322949128189</v>
       </c>
       <c r="N22" t="b">
         <v>1</v>
@@ -1517,28 +1517,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F23" t="n">
-        <v>-19.15161597580796</v>
+        <v>-19.15161053622666</v>
       </c>
       <c r="G23" t="n">
         <v>9</v>
       </c>
       <c r="H23" t="n">
-        <v>-2.127957330645328</v>
+        <v>-2.127956726247406</v>
       </c>
       <c r="I23" t="n">
-        <v>-191516.1597580796</v>
+        <v>-191516.1053622665</v>
       </c>
       <c r="J23" t="n">
-        <v>808483.8402419204</v>
+        <v>808483.8946377335</v>
       </c>
       <c r="K23" t="n">
-        <v>16129.61610352126</v>
+        <v>16129.61622595941</v>
       </c>
       <c r="L23" t="n">
         <v>4.777777777777778</v>
       </c>
       <c r="M23" t="n">
-        <v>19.15161597580796</v>
+        <v>19.15161053622666</v>
       </c>
       <c r="N23" t="b">
         <v>1</v>
@@ -1565,28 +1565,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F24" t="n">
-        <v>-20.08206288359109</v>
+        <v>-20.08205739995612</v>
       </c>
       <c r="G24" t="n">
         <v>9</v>
       </c>
       <c r="H24" t="n">
-        <v>-2.23134032039901</v>
+        <v>-2.231339711106236</v>
       </c>
       <c r="I24" t="n">
-        <v>-200820.6288359109</v>
+        <v>-200820.5739995613</v>
       </c>
       <c r="J24" t="n">
-        <v>799179.3711640891</v>
+        <v>799179.4260004387</v>
       </c>
       <c r="K24" t="n">
-        <v>15998.80948144588</v>
+        <v>15998.80961438033</v>
       </c>
       <c r="L24" t="n">
         <v>5</v>
       </c>
       <c r="M24" t="n">
-        <v>20.08206288359109</v>
+        <v>20.08205739995612</v>
       </c>
       <c r="N24" t="b">
         <v>1</v>
@@ -1613,28 +1613,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>-20.31736015596351</v>
+        <v>-20.3173561389661</v>
       </c>
       <c r="G25" t="n">
         <v>12</v>
       </c>
       <c r="H25" t="n">
-        <v>-1.693113346330293</v>
+        <v>-1.693113011580509</v>
       </c>
       <c r="I25" t="n">
-        <v>-203173.6015596351</v>
+        <v>-203173.561389661</v>
       </c>
       <c r="J25" t="n">
-        <v>796826.3984403649</v>
+        <v>796826.438610339</v>
       </c>
       <c r="K25" t="n">
-        <v>23518.54818965333</v>
+        <v>23518.5460953712</v>
       </c>
       <c r="L25" t="n">
         <v>7.333333333333333</v>
       </c>
       <c r="M25" t="n">
-        <v>30.31090295231158</v>
+        <v>30.31089360613182</v>
       </c>
       <c r="N25" t="b">
         <v>1</v>
@@ -1661,28 +1661,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F26" t="n">
-        <v>-20.31736015596351</v>
+        <v>-20.3173561389661</v>
       </c>
       <c r="G26" t="n">
         <v>12</v>
       </c>
       <c r="H26" t="n">
-        <v>-1.693113346330293</v>
+        <v>-1.693113011580509</v>
       </c>
       <c r="I26" t="n">
-        <v>-203173.6015596351</v>
+        <v>-203173.561389661</v>
       </c>
       <c r="J26" t="n">
-        <v>796826.3984403649</v>
+        <v>796826.438610339</v>
       </c>
       <c r="K26" t="n">
-        <v>23518.54818965333</v>
+        <v>23518.5460953712</v>
       </c>
       <c r="L26" t="n">
         <v>7.333333333333333</v>
       </c>
       <c r="M26" t="n">
-        <v>30.31090295231158</v>
+        <v>30.31089360613182</v>
       </c>
       <c r="N26" t="b">
         <v>1</v>
@@ -1709,28 +1709,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F27" t="n">
-        <v>-20.93488626708447</v>
+        <v>-20.93489075806439</v>
       </c>
       <c r="G27" t="n">
         <v>12</v>
       </c>
       <c r="H27" t="n">
-        <v>-1.744573855590372</v>
+        <v>-1.744574229838699</v>
       </c>
       <c r="I27" t="n">
-        <v>-209348.8626708447</v>
+        <v>-209348.9075806439</v>
       </c>
       <c r="J27" t="n">
-        <v>790651.1373291553</v>
+        <v>790651.0924193561</v>
       </c>
       <c r="K27" t="n">
-        <v>23454.02281004341</v>
+        <v>23454.01982844635</v>
       </c>
       <c r="L27" t="n">
         <v>7.833333333333333</v>
       </c>
       <c r="M27" t="n">
-        <v>30.85098090619993</v>
+        <v>30.85097904615927</v>
       </c>
       <c r="N27" t="b">
         <v>1</v>
@@ -1757,28 +1757,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F28" t="n">
-        <v>-21.0629487189292</v>
+        <v>-21.06291471094706</v>
       </c>
       <c r="G28" t="n">
         <v>18</v>
       </c>
       <c r="H28" t="n">
-        <v>-1.170163817718289</v>
+        <v>-1.170161928385947</v>
       </c>
       <c r="I28" t="n">
-        <v>-210629.487189292</v>
+        <v>-210629.1471094706</v>
       </c>
       <c r="J28" t="n">
-        <v>789370.512810708</v>
+        <v>789370.8528905294</v>
       </c>
       <c r="K28" t="n">
-        <v>32767.49129634228</v>
+        <v>32767.49932306822</v>
       </c>
       <c r="L28" t="n">
         <v>7.388888888888889</v>
       </c>
       <c r="M28" t="n">
-        <v>21.78355491438056</v>
+        <v>21.78352121685293</v>
       </c>
       <c r="N28" t="b">
         <v>1</v>
@@ -1805,28 +1805,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F29" t="n">
-        <v>-21.18977443204955</v>
+        <v>-21.18976381416782</v>
       </c>
       <c r="G29" t="n">
         <v>9</v>
       </c>
       <c r="H29" t="n">
-        <v>-2.354419381338839</v>
+        <v>-2.354418201574202</v>
       </c>
       <c r="I29" t="n">
-        <v>-211897.7443204955</v>
+        <v>-211897.6381416782</v>
       </c>
       <c r="J29" t="n">
-        <v>788102.2556795045</v>
+        <v>788102.3618583218</v>
       </c>
       <c r="K29" t="n">
-        <v>16029.66495572286</v>
+        <v>16029.66577851262</v>
       </c>
       <c r="L29" t="n">
         <v>7.111111111111111</v>
       </c>
       <c r="M29" t="n">
-        <v>21.18977443204955</v>
+        <v>21.18976381416782</v>
       </c>
       <c r="N29" t="b">
         <v>1</v>
@@ -1853,28 +1853,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F30" t="n">
-        <v>-21.18977443204955</v>
+        <v>-21.18976381416782</v>
       </c>
       <c r="G30" t="n">
         <v>9</v>
       </c>
       <c r="H30" t="n">
-        <v>-2.354419381338839</v>
+        <v>-2.354418201574202</v>
       </c>
       <c r="I30" t="n">
-        <v>-211897.7443204955</v>
+        <v>-211897.6381416782</v>
       </c>
       <c r="J30" t="n">
-        <v>788102.2556795045</v>
+        <v>788102.3618583218</v>
       </c>
       <c r="K30" t="n">
-        <v>16029.66495572286</v>
+        <v>16029.66577851262</v>
       </c>
       <c r="L30" t="n">
         <v>7.111111111111111</v>
       </c>
       <c r="M30" t="n">
-        <v>21.18977443204955</v>
+        <v>21.18976381416782</v>
       </c>
       <c r="N30" t="b">
         <v>1</v>
@@ -1901,28 +1901,28 @@
         <v>33.33333333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>-21.48954556589931</v>
+        <v>-21.4895201590767</v>
       </c>
       <c r="G31" t="n">
         <v>18</v>
       </c>
       <c r="H31" t="n">
-        <v>-1.193863642549962</v>
+        <v>-1.193862231059817</v>
       </c>
       <c r="I31" t="n">
-        <v>-214895.4556589931</v>
+        <v>-214895.201590767</v>
       </c>
       <c r="J31" t="n">
-        <v>785104.5443410069</v>
+        <v>785104.798409233</v>
       </c>
       <c r="K31" t="n">
-        <v>32712.28466835502</v>
+        <v>32712.29149185974</v>
       </c>
       <c r="L31" t="n">
         <v>7.777777777777778</v>
       </c>
       <c r="M31" t="n">
-        <v>22.20625741356471</v>
+        <v>22.20623223867772</v>
       </c>
       <c r="N31" t="b">
         <v>1</v>
@@ -1949,28 +1949,28 @@
         <v>22.22222222222222</v>
       </c>
       <c r="F32" t="n">
-        <v>-21.8005394896179</v>
+        <v>-21.8005373380602</v>
       </c>
       <c r="G32" t="n">
         <v>9</v>
       </c>
       <c r="H32" t="n">
-        <v>-2.4222821655131</v>
+        <v>-2.422281926451133</v>
       </c>
       <c r="I32" t="n">
-        <v>-218005.394896179</v>
+        <v>-218005.373380602</v>
       </c>
       <c r="J32" t="n">
-        <v>781994.605103821</v>
+        <v>781994.626619398</v>
       </c>
       <c r="K32" t="n">
-        <v>15956.37122227936</v>
+        <v>15956.3710305271</v>
       </c>
       <c r="L32" t="n">
         <v>7.777777777777778</v>
       </c>
       <c r="M32" t="n">
-        <v>21.8005394896179</v>
+        <v>21.8005373380602</v>
       </c>
       <c r="N32" t="b">
         <v>1</v>
@@ -1997,28 +1997,28 @@
         <v>31.25</v>
       </c>
       <c r="F33" t="n">
-        <v>-22.18246585240811</v>
+        <v>-22.18244374025001</v>
       </c>
       <c r="G33" t="n">
         <v>16</v>
       </c>
       <c r="H33" t="n">
-        <v>-1.386404115775507</v>
+        <v>-1.386402733765626</v>
       </c>
       <c r="I33" t="n">
-        <v>-221824.6585240811</v>
+        <v>-221824.4374025001</v>
       </c>
       <c r="J33" t="n">
-        <v>778175.3414759189</v>
+        <v>778175.5625974999</v>
       </c>
       <c r="K33" t="n">
-        <v>29001.06359338484</v>
+        <v>29001.06904510031</v>
       </c>
       <c r="L33" t="n">
         <v>7.375</v>
       </c>
       <c r="M33" t="n">
-        <v>22.89285211983827</v>
+        <v>22.89283020953921</v>
       </c>
       <c r="N33" t="b">
         <v>1</v>
@@ -2045,28 +2045,28 @@
         <v>20</v>
       </c>
       <c r="F34" t="n">
-        <v>-22.41382466843616</v>
+        <v>-22.4137934282424</v>
       </c>
       <c r="G34" t="n">
         <v>10</v>
       </c>
       <c r="H34" t="n">
-        <v>-2.241382466843616</v>
+        <v>-2.24137934282424</v>
       </c>
       <c r="I34" t="n">
-        <v>-224138.2466843616</v>
+        <v>-224137.934282424</v>
       </c>
       <c r="J34" t="n">
-        <v>775861.7533156384</v>
+        <v>775862.065717576</v>
       </c>
       <c r="K34" t="n">
-        <v>17678.80530903795</v>
+        <v>17678.81033271277</v>
       </c>
       <c r="L34" t="n">
         <v>7.2</v>
       </c>
       <c r="M34" t="n">
-        <v>22.41382466843616</v>
+        <v>22.4137934282424</v>
       </c>
       <c r="N34" t="b">
         <v>1</v>
@@ -2093,28 +2093,28 @@
         <v>27.27272727272727</v>
       </c>
       <c r="F35" t="n">
-        <v>-23.1595426134089</v>
+        <v>-23.15951543006937</v>
       </c>
       <c r="G35" t="n">
         <v>11</v>
       </c>
       <c r="H35" t="n">
-        <v>-2.105412964855355</v>
+        <v>-2.105410493642669</v>
       </c>
       <c r="I35" t="n">
-        <v>-231595.426134089</v>
+        <v>-231595.1543006937</v>
       </c>
       <c r="J35" t="n">
-        <v>768404.573865911</v>
+        <v>768404.8456993063</v>
       </c>
       <c r="K35" t="n">
-        <v>21208.74702497262</v>
+        <v>21208.75056024034</v>
       </c>
       <c r="L35" t="n">
         <v>6</v>
       </c>
       <c r="M35" t="n">
-        <v>29.81029737946523</v>
+        <v>29.81028796620325</v>
       </c>
       <c r="N35" t="b">
         <v>1</v>
@@ -2141,28 +2141,28 @@
         <v>27.27272727272727</v>
       </c>
       <c r="F36" t="n">
-        <v>-23.1595426134089</v>
+        <v>-23.15951543006937</v>
       </c>
       <c r="G36" t="n">
         <v>11</v>
       </c>
       <c r="H36" t="n">
-        <v>-2.105412964855355</v>
+        <v>-2.105410493642669</v>
       </c>
       <c r="I36" t="n">
-        <v>-231595.426134089</v>
+        <v>-231595.1543006937</v>
       </c>
       <c r="J36" t="n">
-        <v>768404.573865911</v>
+        <v>768404.8456993063</v>
       </c>
       <c r="K36" t="n">
-        <v>21208.74702497262</v>
+        <v>21208.75056024034</v>
       </c>
       <c r="L36" t="n">
         <v>6</v>
       </c>
       <c r="M36" t="n">
-        <v>29.81029737946523</v>
+        <v>29.81028796620325</v>
       </c>
       <c r="N36" t="b">
         <v>1</v>
@@ -2189,28 +2189,28 @@
         <v>27.27272727272727</v>
       </c>
       <c r="F37" t="n">
-        <v>-25.4023822564724</v>
+        <v>-25.40237669746409</v>
       </c>
       <c r="G37" t="n">
         <v>11</v>
       </c>
       <c r="H37" t="n">
-        <v>-2.309307477861127</v>
+        <v>-2.309306972496735</v>
       </c>
       <c r="I37" t="n">
-        <v>-254023.822564724</v>
+        <v>-254023.7669746409</v>
       </c>
       <c r="J37" t="n">
-        <v>745976.177435276</v>
+        <v>745976.2330253591</v>
       </c>
       <c r="K37" t="n">
-        <v>20554.5578298803</v>
+        <v>20554.5568458716</v>
       </c>
       <c r="L37" t="n">
         <v>5.727272727272728</v>
       </c>
       <c r="M37" t="n">
-        <v>30.34012956460909</v>
+        <v>30.34012022234575</v>
       </c>
       <c r="N37" t="b">
         <v>1</v>
@@ -2237,28 +2237,28 @@
         <v>27.27272727272727</v>
       </c>
       <c r="F38" t="n">
-        <v>-25.4023822564724</v>
+        <v>-25.40237669746409</v>
       </c>
       <c r="G38" t="n">
         <v>11</v>
       </c>
       <c r="H38" t="n">
-        <v>-2.309307477861127</v>
+        <v>-2.309306972496735</v>
       </c>
       <c r="I38" t="n">
-        <v>-254023.822564724</v>
+        <v>-254023.7669746409</v>
       </c>
       <c r="J38" t="n">
-        <v>745976.177435276</v>
+        <v>745976.2330253591</v>
       </c>
       <c r="K38" t="n">
-        <v>20554.5578298803</v>
+        <v>20554.5568458716</v>
       </c>
       <c r="L38" t="n">
         <v>5.727272727272728</v>
       </c>
       <c r="M38" t="n">
-        <v>30.34012956460909</v>
+        <v>30.34012022234575</v>
       </c>
       <c r="N38" t="b">
         <v>1</v>
@@ -2285,28 +2285,28 @@
         <v>27.27272727272727</v>
       </c>
       <c r="F39" t="n">
-        <v>-25.98050061159245</v>
+        <v>-25.98050303155757</v>
       </c>
       <c r="G39" t="n">
         <v>11</v>
       </c>
       <c r="H39" t="n">
-        <v>-2.361863691962951</v>
+        <v>-2.361863911959779</v>
       </c>
       <c r="I39" t="n">
-        <v>-259805.0061159246</v>
+        <v>-259805.0303155757</v>
       </c>
       <c r="J39" t="n">
-        <v>740194.9938840754</v>
+        <v>740194.9696844243</v>
       </c>
       <c r="K39" t="n">
-        <v>20494.1501715614</v>
+        <v>20494.14835540596</v>
       </c>
       <c r="L39" t="n">
         <v>6.272727272727272</v>
       </c>
       <c r="M39" t="n">
-        <v>30.87998125065678</v>
+        <v>30.87997939139623</v>
       </c>
       <c r="N39" t="b">
         <v>1</v>
@@ -2333,28 +2333,28 @@
         <v>26.66666666666667</v>
       </c>
       <c r="F40" t="n">
-        <v>-26.05075909996263</v>
+        <v>-26.05071665438348</v>
       </c>
       <c r="G40" t="n">
         <v>15</v>
       </c>
       <c r="H40" t="n">
-        <v>-1.736717273330842</v>
+        <v>-1.736714443625565</v>
       </c>
       <c r="I40" t="n">
-        <v>-260507.5909996263</v>
+        <v>-260507.1665438348</v>
       </c>
       <c r="J40" t="n">
-        <v>739492.4090003737</v>
+        <v>739492.8334561652</v>
       </c>
       <c r="K40" t="n">
-        <v>27709.71061597609</v>
+        <v>27709.72013489898</v>
       </c>
       <c r="L40" t="n">
         <v>7.666666666666667</v>
       </c>
       <c r="M40" t="n">
-        <v>30.39518833788895</v>
+        <v>30.39517351812237</v>
       </c>
       <c r="N40" t="b">
         <v>1</v>
@@ -2381,28 +2381,28 @@
         <v>26.66666666666667</v>
       </c>
       <c r="F41" t="n">
-        <v>-26.05075909996263</v>
+        <v>-26.05071665438348</v>
       </c>
       <c r="G41" t="n">
         <v>15</v>
       </c>
       <c r="H41" t="n">
-        <v>-1.736717273330842</v>
+        <v>-1.736714443625565</v>
       </c>
       <c r="I41" t="n">
-        <v>-260507.5909996263</v>
+        <v>-260507.1665438348</v>
       </c>
       <c r="J41" t="n">
-        <v>739492.4090003737</v>
+        <v>739492.8334561652</v>
       </c>
       <c r="K41" t="n">
-        <v>27709.71061597609</v>
+        <v>27709.72013489898</v>
       </c>
       <c r="L41" t="n">
         <v>7.666666666666667</v>
       </c>
       <c r="M41" t="n">
-        <v>30.39518833788895</v>
+        <v>30.39517351812237</v>
       </c>
       <c r="N41" t="b">
         <v>1</v>
@@ -2429,28 +2429,28 @@
         <v>31.57894736842105</v>
       </c>
       <c r="F42" t="n">
-        <v>-26.68750661798311</v>
+        <v>-26.68746596961783</v>
       </c>
       <c r="G42" t="n">
         <v>19</v>
       </c>
       <c r="H42" t="n">
-        <v>-1.404605611472795</v>
+        <v>-1.404603472085149</v>
       </c>
       <c r="I42" t="n">
-        <v>-266875.0661798312</v>
+        <v>-266874.6596961783</v>
       </c>
       <c r="J42" t="n">
-        <v>733124.9338201688</v>
+        <v>733125.3403038217</v>
       </c>
       <c r="K42" t="n">
-        <v>32766.42932660343</v>
+        <v>32766.44092380702</v>
       </c>
       <c r="L42" t="n">
         <v>6.421052631578948</v>
       </c>
       <c r="M42" t="n">
-        <v>27.35676694729234</v>
+        <v>27.35672667000075</v>
       </c>
       <c r="N42" t="b">
         <v>1</v>
@@ -2477,28 +2477,28 @@
         <v>26.66666666666667</v>
       </c>
       <c r="F43" t="n">
-        <v>-29.21699061620166</v>
+        <v>-29.21696315461589</v>
       </c>
       <c r="G43" t="n">
         <v>15</v>
       </c>
       <c r="H43" t="n">
-        <v>-1.947799374413444</v>
+        <v>-1.94779754364106</v>
       </c>
       <c r="I43" t="n">
-        <v>-292169.9061620166</v>
+        <v>-292169.6315461589</v>
       </c>
       <c r="J43" t="n">
-        <v>707830.0938379834</v>
+        <v>707830.3684538411</v>
       </c>
       <c r="K43" t="n">
-        <v>27306.48110221214</v>
+        <v>27306.48888194328</v>
       </c>
       <c r="L43" t="n">
         <v>8.133333333333333</v>
       </c>
       <c r="M43" t="n">
-        <v>33.37540754885243</v>
+        <v>33.37540575671638</v>
       </c>
       <c r="N43" t="b">
         <v>1</v>
@@ -2525,28 +2525,28 @@
         <v>21.42857142857143</v>
       </c>
       <c r="F44" t="n">
-        <v>-33.00990746680639</v>
+        <v>-33.00988647658523</v>
       </c>
       <c r="G44" t="n">
         <v>14</v>
       </c>
       <c r="H44" t="n">
-        <v>-2.357850533343314</v>
+        <v>-2.357849034041802</v>
       </c>
       <c r="I44" t="n">
-        <v>-330099.0746680639</v>
+        <v>-330098.8647658523</v>
       </c>
       <c r="J44" t="n">
-        <v>669900.9253319361</v>
+        <v>669901.1352341477</v>
       </c>
       <c r="K44" t="n">
-        <v>24901.6694524773</v>
+        <v>24901.67272652376</v>
       </c>
       <c r="L44" t="n">
         <v>5.071428571428571</v>
       </c>
       <c r="M44" t="n">
-        <v>33.47858667145973</v>
+        <v>33.4785777501029</v>
       </c>
       <c r="N44" t="b">
         <v>1</v>
@@ -2573,28 +2573,28 @@
         <v>21.42857142857143</v>
       </c>
       <c r="F45" t="n">
-        <v>-33.00990746680639</v>
+        <v>-33.00988647658523</v>
       </c>
       <c r="G45" t="n">
         <v>14</v>
       </c>
       <c r="H45" t="n">
-        <v>-2.357850533343314</v>
+        <v>-2.357849034041802</v>
       </c>
       <c r="I45" t="n">
-        <v>-330099.0746680639</v>
+        <v>-330098.8647658523</v>
       </c>
       <c r="J45" t="n">
-        <v>669900.9253319361</v>
+        <v>669901.1352341477</v>
       </c>
       <c r="K45" t="n">
-        <v>24901.6694524773</v>
+        <v>24901.67272652376</v>
       </c>
       <c r="L45" t="n">
         <v>5.071428571428571</v>
       </c>
       <c r="M45" t="n">
-        <v>33.47858667145973</v>
+        <v>33.4785777501029</v>
       </c>
       <c r="N45" t="b">
         <v>1</v>
@@ -2621,28 +2621,28 @@
         <v>21.42857142857143</v>
       </c>
       <c r="F46" t="n">
-        <v>-33.52906884589738</v>
+        <v>-33.52905514493179</v>
       </c>
       <c r="G46" t="n">
         <v>14</v>
       </c>
       <c r="H46" t="n">
-        <v>-2.39493348899267</v>
+        <v>-2.394932510352271</v>
       </c>
       <c r="I46" t="n">
-        <v>-335290.6884589738</v>
+        <v>-335290.5514493178</v>
       </c>
       <c r="J46" t="n">
-        <v>664709.3115410262</v>
+        <v>664709.4485506822</v>
       </c>
       <c r="K46" t="n">
-        <v>24833.34312100902</v>
+        <v>24833.34543720668</v>
       </c>
       <c r="L46" t="n">
         <v>5.5</v>
       </c>
       <c r="M46" t="n">
-        <v>33.99411586953651</v>
+        <v>33.99411409404306</v>
       </c>
       <c r="N46" t="b">
         <v>1</v>

</xml_diff>